<commit_message>
Update analysis files and documentation for Dalarna University courses
- Modified multiple Excel files related to course analysis, including examinations, grading scales, and terminology across various programs (IHV, IKS, ISLL).
- Updated Markdown documentation for prerequisite requirements, reflecting changes in the number of problematic course plans and adding new entries for unknown courses.
- Adjusted download links and counts in the documentation to match the updated Excel files.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -472,34 +472,34 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>GIK2XJ</t>
+          <t>BY1059</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Refererar okänd HDa-kurs</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Osannolikt kort (22 tecken): '- Programmering 7,5 hp'</t>
+          <t>Refererad kurs hittas ej i vaulten: 'Byggprojekt småhus'</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GIK2XZ</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -509,24 +509,24 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Refererar okänd HDa-kurs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Osannolikt kort (22 tecken): '- Databassystem 7,5 hp'</t>
+          <t>Refererad kurs hittas ej i vaulten: 'Introduktion till Informatik och eTjänster'</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IK1032</t>
+          <t>GIK2XJ</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -536,29 +536,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Stor sv/en-längdskillnad</t>
+          <t>Osannolikt kort innehåll</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Längdskillnad sv 121 tecken vs en 32 tecken (×3.8)</t>
+          <t>Osannolikt kort (22 tecken): '- Programmering 7,5 hp'</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XJ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>GMD2GF</t>
+          <t>GIK2XZ</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -568,73 +568,73 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
+          <t>Osannolikt kort (22 tecken): '- Databassystem 7,5 hp'</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2XZ</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GMD2GG</t>
+          <t>IK1032</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Stor sv/en-längdskillnad</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
+          <t>Längdskillnad sv 121 tecken vs en 32 tecken (×3.8)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>GMD2H3</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Refererar okänd HDa-kurs</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Osannolikt kort (16 tecken): '- Algebra 7,5 hp'</t>
+          <t>Refererad kurs hittas ej i vaulten: 'Java - Grafiska användargränssnitt med Swing'</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>GMD2H5</t>
+          <t>GMD2GF</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -649,19 +649,19 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Osannolikt kort (16 tecken): '- Algebra 7,5 hp'</t>
+          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>GMD2GG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -671,24 +671,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Stor sv/en-längdskillnad</t>
+          <t>Osannolikt kort innehåll</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Längdskillnad sv 87 tecken vs en 199 tecken (×2.3)</t>
+          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2GG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GMD2MH</t>
+          <t>GMD2H3</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -708,14 +708,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H3</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GMD2MJ</t>
+          <t>GMD2H5</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -735,14 +735,14 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2H5</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>GMD2XQ</t>
+          <t>GMD2HG</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -752,29 +752,29 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Stor sv/en-längdskillnad</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
+          <t>Längdskillnad sv 87 tecken vs en 199 tecken (×2.3)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AEG2AX</t>
+          <t>GMD2MH</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -784,24 +784,24 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Osannolikt kort (21 tecken): '- Solcellsteknik 5 hp'</t>
+          <t>Osannolikt kort (16 tecken): '- Algebra 7,5 hp'</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MH</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GEG38F</t>
+          <t>GMD2MJ</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -811,24 +811,24 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Osannolikt kort (19 tecken): '- Byggfysik, 7,5 hp'</t>
+          <t>Osannolikt kort (16 tecken): '- Algebra 7,5 hp'</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG38F</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2MJ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GEG39Y</t>
+          <t>GMD2XQ</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -838,46 +838,46 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Osannolikt kort (16 tecken): '- Ellära, 7,5 hp'</t>
+          <t>Osannolikt kort (13 tecken): '- Lärarexamen'</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2XQ</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GEG39Z</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Refererar okänd HDa-kurs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Osannolikt kort (23 tecken): '- Elkraftteknik, 7,5 hp'</t>
+          <t>Refererad kurs hittas ej i vaulten: 'Mekanik grundläggande kurs'</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GEG3A2</t>
+          <t>AEG2AX</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -892,19 +892,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Osannolikt kort (16 tecken): '- Ellära, 7,5 hp'</t>
+          <t>Osannolikt kort (21 tecken): '- Solcellsteknik 5 hp'</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3A2</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AEG2AX</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>GEG3BX</t>
+          <t>EG1012</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -914,24 +914,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Osannolikt kort innehåll</t>
+          <t>Refererar okänd HDa-kurs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Osannolikt kort (23 tecken): '- Elkraftteknik, 7,5 hp'</t>
+          <t>Refererad kurs hittas ej i vaulten: 'Mekanik för energiingenjörer'</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3BX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>GEG3DU</t>
+          <t>GEG38F</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -946,44 +946,179 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Osannolikt kort (22 tecken): '- Termodynamik, 7,5 hp'</t>
+          <t>Osannolikt kort (19 tecken): '- Byggfysik, 7,5 hp'</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3DU</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG38F</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>GEG39Y</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Osannolikt kort (16 tecken): '- Ellära, 7,5 hp'</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>GEG39Z</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Osannolikt kort (23 tecken): '- Elkraftteknik, 7,5 hp'</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG39Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>GEG3A2</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Osannolikt kort (16 tecken): '- Ellära, 7,5 hp'</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3A2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>GEG3BX</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Osannolikt kort (23 tecken): '- Elkraftteknik, 7,5 hp'</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3BX</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>GEG3DU</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Osannolikt kort (22 tecken): '- Termodynamik, 7,5 hp'</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3DU</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>GEG3FY</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>MÖY</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Osannolikt kort innehåll</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Osannolikt kort innehåll</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
         <is>
           <t>Osannolikt kort (22 tecken): '- 60 hp i energiteknik'</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="E25" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GEG3FY</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E20"/>
+  <autoFilter ref="A1:E25"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1023,6 +1158,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update course offerings across multiple language programs, expanding course lists and adding new courses in English, French, Italian, Japanese, Chinese, Portuguese, Russian, Spanish, Swedish, Swedish as a second language, and German. Adjusted the number of inactive course plans accordingly.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -526,7 +526,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IK1032</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -536,29 +536,29 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Stor sv/en-längdskillnad</t>
+          <t>Refererar troligen nedlagd kurs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Längdskillnad sv 121 tecken vs en 32 tecken (×3.8)</t>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Java - Grafiska användargränssnitt med Swing'</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1032</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -568,98 +568,44 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Java - Grafiska användargränssnitt med Swing'</t>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GMD2HG</t>
+          <t>EG1012</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Stor sv/en-längdskillnad</t>
+          <t>Refererar troligen nedlagd kurs</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Längdskillnad sv 87 tecken vs en 199 tecken (×2.3)</t>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik för energiingenjörer'</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMD2HG</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>MT1060</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>MTA</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Refererar troligen nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>EG1012</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>MÖY</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Refererar troligen nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik för energiingenjörer'</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E8"/>
+  <autoFilter ref="A1:E6"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -671,10 +617,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add analysis of discontinued course references for ISLL program
- Created a new Markdown file for documenting problematic educational plans and their discontinued courses.
- Added an Excel file containing detailed references to discontinued courses for the ISLL program.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -499,113 +499,815 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>BY1059</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Introduktion till Informatik och eTjänster'</t>
+          <t>`Byggprojekt småhus` → `BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>BY2022</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Java - Grafiska användargränssnitt med Swing'</t>
+          <t>`Energiteknik` → `EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>BY2022</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>BYA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
+          <t>`Byggprojekt stora byggnader` → `GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>GBY3AX</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>BYA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>`Byggstatik` → `BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ET1029</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ETA</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>`Programmeringsteknik` → `DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>FY1018</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FYA</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>`Linjär algebra för ingenjörer` → `MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>FY1018</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>FYA</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>`Envariabelanalys för ingenjörer` → `MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>GIE2MF</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>GIE36Y</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>IE1069</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>IEA</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>AIK232</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>GIK23M</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>GIK2PD</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Refererar troligen nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Introduktion till Informatik och eTjänster'</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>GIK2PD</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>`Introduktion till Informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>GIK32L</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>`Layout` → `GT1021` (nedlagd 2014-06-16); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32L</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>IK1064</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Refererar troligen nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Java - Grafiska användargränssnitt med Swing'</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>IK1064</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>`Java - Grafiska användargränssnitt med Swing` → `IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>IK1066</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>IKA</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>`Introduktion till informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>AMD238</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>MDI</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>AMD239</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>MDI</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>MT1060</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>MTA</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Refererar troligen nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
           <t>EG1012</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>MÖY</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Refererar troligen nedlagd kurs</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik för energiingenjörer'</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>EG1012</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>MÖY</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>`Mekanik för energiingenjörer` → `GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>`Arkitektur` → `BY1048` (nedlagd 2015-09-23); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>`Fysisk planering` → `GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>GSQ23K</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>GSQ25K</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>GSQ25K</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SQQ</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>`Transportplanering` → `GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>GMI23G</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>GMI26H</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>XYZ</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Refererar bekräftat nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E6"/>
+  <autoFilter ref="A1:E32"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -617,6 +1319,58 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis files across multiple courses
- Updated various Excel files related to course analysis for IIT, IHV, IKS, and ISLL programs, reflecting changes in course references and requirements.
- Modified Markdown files to reflect updated download links and counts for prerequisite requirements.
- Ensured consistency in naming and formatting across all updated documents.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$E$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E32"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -482,12 +482,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Byggprojekt småhus'</t>
+          <t>`Byggprojekt småhus` → `BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -499,7 +499,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>BY1059</t>
+          <t>BY2022</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -514,12 +514,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>`Byggprojekt småhus` → `BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
+          <t>`Energiteknik` → `EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
       </c>
     </row>
@@ -541,7 +541,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>`Energiteknik` → `EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
+          <t>`Byggprojekt stora byggnader` → `GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -553,7 +553,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>BY2022</t>
+          <t>GBY3AX</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -568,24 +568,24 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`Byggprojekt stora byggnader` → `GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
+          <t>`Byggstatik` → `BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>GBY3AX</t>
+          <t>ET1029</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BYA</t>
+          <t>ETA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -595,24 +595,24 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>`Byggstatik` → `BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
+          <t>`Programmeringsteknik` → `DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ET1029</t>
+          <t>FY1018</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ETA</t>
+          <t>FYA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -622,12 +622,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>`Programmeringsteknik` → `DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
+          <t>`Linjär algebra för ingenjörer` → `MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
         </is>
       </c>
     </row>
@@ -649,7 +649,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>`Linjär algebra för ingenjörer` → `MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
+          <t>`Envariabelanalys för ingenjörer` → `MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -661,12 +661,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>FY1018</t>
+          <t>GIE2MF</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>FYA</t>
+          <t>IEA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -676,19 +676,19 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>`Envariabelanalys för ingenjörer` → `MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
+          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>GIE2MF</t>
+          <t>GIE36Y</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -708,14 +708,14 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Y</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>GIE36Y</t>
+          <t>IE1069</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -735,19 +735,19 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Y</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>IE1069</t>
+          <t>AIK232</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>IEA</t>
+          <t>IKA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -757,19 +757,19 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>AIK232</t>
+          <t>GIK23M</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -789,14 +789,14 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>GIK23M</t>
+          <t>GIK2PD</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -811,19 +811,19 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till Informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>GIK32L</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,24 +833,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Introduktion till Informatik och eTjänster'</t>
+          <t>`Layout` → `GT1021` (nedlagd 2014-06-16); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32L</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>GIK2PD</t>
+          <t>IK1064</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -865,19 +865,19 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>`Introduktion till Informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>`Java - Grafiska användargränssnitt med Swing` → `IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>GIK32L</t>
+          <t>IK1066</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -892,51 +892,51 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>`Layout` → `GT1021` (nedlagd 2014-06-16); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK32L</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>AMD238</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Java - Grafiska användargränssnitt med Swing'</t>
+          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>IK1064</t>
+          <t>AMD239</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MDI</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -946,51 +946,51 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>`Java - Grafiska användargränssnitt med Swing` → `IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>IK1066</t>
+          <t>MT1060</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>IKA</t>
+          <t>MTA</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
+          <t>Refererar troligen nedlagd kurs</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>`Introduktion till informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>AMD238</t>
+          <t>EG1012</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>MÖY</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1000,24 +1000,24 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+          <t>`Mekanik för energiingenjörer` → `GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD238</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>AMD239</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>MDI</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1027,78 +1027,78 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>`Vetenskapsteori` → `GPG263` (nedlagd 2024-03-25); förkunskap nämner nedlagd kurs</t>
+          <t>`Arkitektur` → `BY1048` (nedlagd 2015-09-23); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AMD239</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>MT1060</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MTA</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
+          <t>`Fysisk planering` → `GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>EG1012</t>
+          <t>GSQ23K</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Refererar troligen nedlagd kurs</t>
+          <t>Refererar bekräftat nedlagd kurs</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik för energiingenjörer'</t>
+          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>EG1012</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MÖY</t>
+          <t>SQQ</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1108,19 +1108,19 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>`Mekanik för energiingenjörer` → `GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GSQ25K</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1135,24 +1135,24 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>`Arkitektur` → `BY1048` (nedlagd 2015-09-23); förkunskap nämner nedlagd kurs</t>
+          <t>`Transportplanering` → `GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GMI23G</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1162,24 +1162,24 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>`Fysisk planering` → `GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
+          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>GSQ23K</t>
+          <t>GMI26H</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>SQQ</t>
+          <t>XYZ</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1189,125 +1189,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>GSQ25K</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>GSQ25K</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>SQQ</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>`Transportplanering` → `GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>GMI23G</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="inlineStr">
-        <is>
-          <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>GMI26H</t>
-        </is>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>XYZ</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>Refererar bekräftat nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
-        </is>
-      </c>
-      <c r="E32" s="2" t="inlineStr">
-        <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E32"/>
+  <autoFilter ref="A1:E28"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1363,14 +1255,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update analysis spreadsheets with new data: Stavfel och språkbruk.xlsx and Övrigt.xlsx
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Förkunskapskrav" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$G$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Förkunskapskrav'!$A$1:$H$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -441,7 +441,8 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
     <col width="70" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="7" max="7"/>
+    <col width="70" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -477,6 +478,11 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>Förslag</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>Länk</t>
         </is>
       </c>
@@ -508,7 +514,12 @@
           <t>`Byggprojekt småhus` → `BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>`BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY1059</t>
         </is>
@@ -541,7 +552,12 @@
           <t>`Energiteknik` → `EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>`EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
@@ -574,7 +590,12 @@
           <t>`Byggprojekt stora byggnader` → `GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>`GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=BY2022</t>
         </is>
@@ -607,7 +628,12 @@
           <t>`Byggstatik` → `BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>`BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GBY3AX</t>
         </is>
@@ -640,7 +666,12 @@
           <t>`Programmeringsteknik` → `DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>`DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=ET1029</t>
         </is>
@@ -673,7 +704,12 @@
           <t>`Linjär algebra för ingenjörer` → `MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>`MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
         </is>
@@ -706,7 +742,12 @@
           <t>`Envariabelanalys för ingenjörer` → `MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>`MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=FY1018</t>
         </is>
@@ -739,7 +780,12 @@
           <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>`IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE2MF</t>
         </is>
@@ -772,7 +818,12 @@
           <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>`IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIE36Y</t>
         </is>
@@ -805,7 +856,12 @@
           <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>`IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IE1069</t>
         </is>
@@ -838,7 +894,12 @@
           <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>`MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=AIK232</t>
         </is>
@@ -871,7 +932,12 @@
           <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>`MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK23M</t>
         </is>
@@ -904,7 +970,12 @@
           <t>`Introduktion till Informatik och eTjänster` → `IK1078` (nedlagd 2022-06-23); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>`IK1078` (nedlagd 2022-06-23); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GIK2PD</t>
         </is>
@@ -941,7 +1012,12 @@
           <t>`Java - Grafiska användargränssnitt med Swing` → `IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>`IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1064</t>
         </is>
@@ -974,7 +1050,12 @@
           <t>`Introduktion till informatik och IT` → `IK1082` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>`IK1082` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
@@ -1007,7 +1088,12 @@
           <t>`Introduktion till informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>`IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=IK1066</t>
         </is>
@@ -1040,7 +1126,8 @@
           <t>Refererad kurs hittas ej i vaulten (troligen nedlagd): 'Mekanik grundläggande kurs'</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1060</t>
         </is>
@@ -1073,7 +1160,12 @@
           <t>`Introduktion till mekanik och hållfasthetslära` → `MT1067` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>`MT1067` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=MT1074</t>
         </is>
@@ -1106,7 +1198,12 @@
           <t>`Mekanik för energiingenjörer` → `GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>`GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=EG1012</t>
         </is>
@@ -1139,7 +1236,12 @@
           <t>`Fysisk planering` → `GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>`GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
@@ -1172,7 +1274,12 @@
           <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>`GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ23K</t>
         </is>
@@ -1205,7 +1312,12 @@
           <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>`GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
@@ -1238,7 +1350,12 @@
           <t>`Transportplanering` → `GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>`GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GSQ25K</t>
         </is>
@@ -1271,7 +1388,12 @@
           <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>`MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI23G</t>
         </is>
@@ -1304,65 +1426,70 @@
           <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>`MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/kurser/kursplan/?code=GMI26H</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G26"/>
+  <autoFilter ref="A1:H26"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H2" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H3" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H4" r:id="rId6"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H5" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H7" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H8" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId18"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId28"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H18" r:id="rId34"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H19" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H21" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H22" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H23" r:id="rId44"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H24" r:id="rId46"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H25" r:id="rId48"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H26" r:id="rId50"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update various analysis files and references in the Dalarna University vault
- Modified content in "Nedlagda kursreferenser.md" to improve clarity and structure of course references.
- Updated multiple Excel files including "Färkunskapskrav.xlsx", "Introfras.xlsx", "Nedlagda kursreferenser.xlsx", "Omfång på lärandemål.xlsx", "Programkurser olänkade.xlsx", "Samstämmighet svenska och engelska.xlsx", "Stavfel och språkbruk.xlsx", and "Övrigt.xlsx" to reflect recent changes and corrections.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Förkunskapskrav.xlsx
@@ -511,7 +511,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>`Byggprojekt småhus` → `BY1055` (nedlagd 2022-04-27); förkunskap nämner nedlagd kurs</t>
+          <t>`Byggprojekt småhus`</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>`Energiteknik` → `EG1000` (nedlagd 2024-05-13); förkunskap nämner nedlagd kurs</t>
+          <t>`Energiteknik`</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -587,7 +587,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>`Byggprojekt stora byggnader` → `GBY24K` (nedlagd 2023-09-28); förkunskap nämner nedlagd kurs</t>
+          <t>`Byggprojekt stora byggnader`</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>`Byggstatik` → `BYB010` (nedlagd 2007-10-22); förkunskap nämner nedlagd kurs</t>
+          <t>`Byggstatik`</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -663,7 +663,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>`Programmeringsteknik` → `DT1043` (nedlagd 2018-09-18); förkunskap nämner nedlagd kurs</t>
+          <t>`Programmeringsteknik`</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -701,7 +701,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>`Linjär algebra för ingenjörer` → `MA1038` (nedlagd 2019-04-02); förkunskap nämner nedlagd kurs</t>
+          <t>`Linjär algebra för ingenjörer`</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -739,7 +739,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>`Envariabelanalys för ingenjörer` → `MA1039` (nedlagd 2019-09-05); förkunskap nämner nedlagd kurs</t>
+          <t>`Envariabelanalys för ingenjörer`</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -777,7 +777,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Industriell ekonomi med kalkylering`</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Industriell ekonomi med kalkylering`</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>`Industriell ekonomi med kalkylering` → `IE1062` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Industriell ekonomi med kalkylering`</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering`</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -929,7 +929,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering`</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -967,7 +967,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>`Introduktion till Informatik och eTjänster` → `IK1078` (nedlagd 2022-06-23); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till Informatik och eTjänster`</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>`Java - Grafiska användargränssnitt med Swing` → `IK1004` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>`Java - Grafiska användargränssnitt med Swing`</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>`Introduktion till informatik och IT` → `IK1082` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till informatik och IT`</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>`Introduktion till informatik` → `IK1016` (nedlagd 2020-06-11); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till informatik`</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1157,7 +1157,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>`Introduktion till mekanik och hållfasthetslära` → `MT1067` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Introduktion till mekanik och hållfasthetslära`</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1195,7 +1195,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>`Mekanik för energiingenjörer` → `GMT2KD` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Mekanik för energiingenjörer`</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1233,7 +1233,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>`Fysisk planering` → `GSQ25G` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Fysisk planering`</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1271,7 +1271,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Regional planering`</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>`Regional planering` → `GSQ25H` (nedlagd 2025-12-08); förkunskap nämner nedlagd kurs</t>
+          <t>`Regional planering`</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1347,7 +1347,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>`Transportplanering` → `GMI22F` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Transportplanering`</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1385,7 +1385,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering`</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>`Grundläggande programmering` → `MI1001` (nedlagd 2024-11-06); förkunskap nämner nedlagd kurs</t>
+          <t>`Grundläggande programmering`</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">

</xml_diff>